<commit_message>
chore: add fixtures, update gitignore, remove debug scripts
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/telepharmacy-selector-discovery/Telepharmacy_CMS_Selectors.xlsx
+++ b/telepharmacy-selector-discovery/Telepharmacy_CMS_Selectors.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Supervisor + Home" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Code Snippets" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Summary" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Chat Page" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -88,7 +89,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="25">
     <fill>
       <patternFill/>
     </fill>
@@ -175,6 +176,41 @@
         <fgColor rgb="00FAFAFA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8EAF6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCCBC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B71C1C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F8E9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -202,7 +238,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -304,6 +340,33 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3701,4 +3764,1298 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>Telepharmacy CMS — Chat Page Selectors  (ยืนยันจาก DOM inspection 2026-06-25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Chat Zone: /home (split-panel) | Zone 1=Queue List | Zone 2=Chat | Zone 3=Patient Info | Zone 4=Prescription | Zone 5=POS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>หมวด</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Element / ฟีเจอร์</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Selector (Playwright / CSS)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Tag จริง</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Class จริง (ตัดสั้น)</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>สถานะ</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>หมายเหตุ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  LAYOUT  (Grid 5 Columns)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="40" t="inlineStr">
+        <is>
+          <t>Layout</t>
+        </is>
+      </c>
+      <c r="B5" s="40" t="inlineStr">
+        <is>
+          <t>Root container</t>
+        </is>
+      </c>
+      <c r="C5" s="40" t="inlineStr">
+        <is>
+          <t>div[class*='h-screen'][class*='flex-col']</t>
+        </is>
+      </c>
+      <c r="D5" s="40" t="inlineStr">
+        <is>
+          <t>div</t>
+        </is>
+      </c>
+      <c r="E5" s="40" t="inlineStr">
+        <is>
+          <t>h-screen flex flex-col bg-slate-100 relative</t>
+        </is>
+      </c>
+      <c r="F5" s="40" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G5" s="40" t="inlineStr">
+        <is>
+          <t>wrapper ทั้งหน้า</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="40" t="inlineStr">
+        <is>
+          <t>Layout</t>
+        </is>
+      </c>
+      <c r="B6" s="40" t="inlineStr">
+        <is>
+          <t>Grid 5 cols</t>
+        </is>
+      </c>
+      <c r="C6" s="40" t="inlineStr">
+        <is>
+          <t>div[class*='grid-cols']</t>
+        </is>
+      </c>
+      <c r="D6" s="40" t="inlineStr">
+        <is>
+          <t>div</t>
+        </is>
+      </c>
+      <c r="E6" s="40" t="inlineStr">
+        <is>
+          <t>h-full grid grid-cols-[300px_1fr_1fr_2fr] gap-0</t>
+        </is>
+      </c>
+      <c r="F6" s="40" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G6" s="40" t="inlineStr">
+        <is>
+          <t>Zone1=300px, Zone2=1fr, Zone3=1fr, Zone4=2fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="40" t="inlineStr">
+        <is>
+          <t>Layout</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="inlineStr">
+        <is>
+          <t>Zone 1 – Queue List panel</t>
+        </is>
+      </c>
+      <c r="C7" s="40" t="inlineStr">
+        <is>
+          <t>div[class*='bg-white'][class*='flex-col'][class*='overflow-hidden']:first-child</t>
+        </is>
+      </c>
+      <c r="D7" s="40" t="inlineStr">
+        <is>
+          <t>div</t>
+        </is>
+      </c>
+      <c r="E7" s="40" t="inlineStr">
+        <is>
+          <t>border-r border-slate-200 bg-white flex flex-col overflow-hidden</t>
+        </is>
+      </c>
+      <c r="F7" s="40" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G7" s="40" t="inlineStr">
+        <is>
+          <t>คอลัมน์ซ้ายสุด — รายการคิวผู้ป่วย</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="40" t="inlineStr">
+        <is>
+          <t>Layout</t>
+        </is>
+      </c>
+      <c r="B8" s="40" t="inlineStr">
+        <is>
+          <t>Zone 2 – Chat panel</t>
+        </is>
+      </c>
+      <c r="C8" s="40" t="inlineStr">
+        <is>
+          <t>div[class*='bg-slate-50'][class*='flex-col'][class*='overflow-hidden']</t>
+        </is>
+      </c>
+      <c r="D8" s="40" t="inlineStr">
+        <is>
+          <t>div</t>
+        </is>
+      </c>
+      <c r="E8" s="40" t="inlineStr">
+        <is>
+          <t>border-r border-slate-200 bg-slate-50 flex flex-col overflow-hidden</t>
+        </is>
+      </c>
+      <c r="F8" s="40" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G8" s="40" t="inlineStr">
+        <is>
+          <t>คอลัมน์ chat messages</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ZONE 1 — QUEUE LIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Zone 1</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Patient card (clickable row)</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>div.flex.items-start.gap-3</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>div</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>flex items-start gap-3</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>คลิกเพื่อเปิด chat ใน Zone 2 — URL ยังอยู่ที่ /home</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Zone 1</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Queue scrollable list</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>div[class*='scrollbar-thin'][class*='space-y-2']</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>div</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>scrollbar-thin flex-1 space-y-2 overflow-y-auto bg-slate-50/40 p-3</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>container ของ patient cards</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Zone 1</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Status badge — WAITING</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>span:has-text('WAITING')</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>span</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>(dynamic — badge text)</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Zone 1</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Status badge — ACTIVE</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>span:has-text('ACTIVE')</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>span</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>(dynamic — badge text)</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Zone 1</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>Status badge — CLOSED</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>span:has-text('CLOSED')</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>span</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>(dynamic — badge text)</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>ปรากฏหลัง Close Encounter</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Zone 1</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>Status badge — PAUSED</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>span:has-text('PAUSED')</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>span</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>(dynamic — badge text)</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>ปรากฏหลัง Pause</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ZONE 2 — CHAT HEADER</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="41" t="inlineStr">
+        <is>
+          <t>Chat Header</t>
+        </is>
+      </c>
+      <c r="B17" s="41" t="inlineStr">
+        <is>
+          <t>Encounter ID ('Encounter #47')</t>
+        </is>
+      </c>
+      <c r="C17" s="41" t="inlineStr">
+        <is>
+          <t>div:has-text('Encounter #')</t>
+        </is>
+      </c>
+      <c r="D17" s="41" t="inlineStr">
+        <is>
+          <t>div</t>
+        </is>
+      </c>
+      <c r="E17" s="41" t="inlineStr">
+        <is>
+          <t>(container ที่มีข้อความ 'Encounter #XX')</t>
+        </is>
+      </c>
+      <c r="F17" s="41" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G17" s="41" t="inlineStr">
+        <is>
+          <t>ข้อความจริงใน header: 'Encounter #47'</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="42" t="inlineStr">
+        <is>
+          <t>Chat Header</t>
+        </is>
+      </c>
+      <c r="B18" s="42" t="inlineStr">
+        <is>
+          <t>Encounter timestamp (14:42)</t>
+        </is>
+      </c>
+      <c r="C18" s="42" t="inlineStr">
+        <is>
+          <t>div[class*='text-slate-400'][class*='text-[11px]']</t>
+        </is>
+      </c>
+      <c r="D18" s="42" t="inlineStr">
+        <is>
+          <t>div</t>
+        </is>
+      </c>
+      <c r="E18" s="42" t="inlineStr">
+        <is>
+          <t>text-[11px] text-slate-400 (approximate)</t>
+        </is>
+      </c>
+      <c r="F18" s="42" t="inlineStr">
+        <is>
+          <t>⚠️ ตรวจเพิ่ม</t>
+        </is>
+      </c>
+      <c r="G18" s="42" t="inlineStr">
+        <is>
+          <t>อาจตรวจด้วย body text regex: /\d{1,2}:\d{2}\s*น\./</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="41" t="inlineStr">
+        <is>
+          <t>Chat Header</t>
+        </is>
+      </c>
+      <c r="B19" s="41" t="inlineStr">
+        <is>
+          <t>Pause button</t>
+        </is>
+      </c>
+      <c r="C19" s="41" t="inlineStr">
+        <is>
+          <t>button:has-text('Pause')</t>
+        </is>
+      </c>
+      <c r="D19" s="41" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="E19" s="41" t="inlineStr">
+        <is>
+          <t>flex h-9 flex-1 items-center justify-center gap-1.5 rounded-lg border border-sla…</t>
+        </is>
+      </c>
+      <c r="F19" s="41" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G19" s="41" t="inlineStr">
+        <is>
+          <t>ปุ่มซ้าย ใน bottom bar ของ Zone 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="41" t="inlineStr">
+        <is>
+          <t>Chat Header</t>
+        </is>
+      </c>
+      <c r="B20" s="41" t="inlineStr">
+        <is>
+          <t>Close Encounter button</t>
+        </is>
+      </c>
+      <c r="C20" s="41" t="inlineStr">
+        <is>
+          <t>button:has-text('Close Encounter')</t>
+        </is>
+      </c>
+      <c r="D20" s="41" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="E20" s="41" t="inlineStr">
+        <is>
+          <t>flex h-9 flex-1 items-center justify-center gap-1.5 rounded-lg text-xs … (สีแดง)</t>
+        </is>
+      </c>
+      <c r="F20" s="41" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G20" s="41" t="inlineStr">
+        <is>
+          <t>ปุ่มขวา — สีแดง</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ZONE 2 — MESSAGE AREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>Message Area</t>
+        </is>
+      </c>
+      <c r="B22" s="41" t="inlineStr">
+        <is>
+          <t>Scrollable message container</t>
+        </is>
+      </c>
+      <c r="C22" s="41" t="inlineStr">
+        <is>
+          <t>div[class*='scrollbar-thin'][class*='space-y-3']</t>
+        </is>
+      </c>
+      <c r="D22" s="41" t="inlineStr">
+        <is>
+          <t>div</t>
+        </is>
+      </c>
+      <c r="E22" s="41" t="inlineStr">
+        <is>
+          <t>scrollbar-thin flex-1 space-y-3 overflow-y-auto bg-slate-50 p-4</t>
+        </is>
+      </c>
+      <c r="F22" s="41" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G22" s="41" t="inlineStr">
+        <is>
+          <t>container ที่บรรจุ message bubbles</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="41" t="inlineStr">
+        <is>
+          <t>Message Area</t>
+        </is>
+      </c>
+      <c r="B23" s="41" t="inlineStr">
+        <is>
+          <t>Date badge divider</t>
+        </is>
+      </c>
+      <c r="C23" s="41" t="inlineStr">
+        <is>
+          <t>div[class*='rounded-full'][class*='ring-1']</t>
+        </is>
+      </c>
+      <c r="D23" s="41" t="inlineStr">
+        <is>
+          <t>div</t>
+        </is>
+      </c>
+      <c r="E23" s="41" t="inlineStr">
+        <is>
+          <t>rounded-full bg-white px-3 py-1 text-[11px] font-medium text-slate-500 ring-1 ring-slate-200</t>
+        </is>
+      </c>
+      <c r="F23" s="41" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G23" s="41" t="inlineStr">
+        <is>
+          <t>แสดงวันที่กั้นกลาง เช่น '25 มิ.ย. 2569'</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="41" t="inlineStr">
+        <is>
+          <t>Message Area</t>
+        </is>
+      </c>
+      <c r="B24" s="41" t="inlineStr">
+        <is>
+          <t>Outbound bubble (operator)</t>
+        </is>
+      </c>
+      <c r="C24" s="41" t="inlineStr">
+        <is>
+          <t>div[class*='justify-end'] div[class*='bg-brand-600']</t>
+        </is>
+      </c>
+      <c r="D24" s="41" t="inlineStr">
+        <is>
+          <t>div</t>
+        </is>
+      </c>
+      <c r="E24" s="41" t="inlineStr">
+        <is>
+          <t>rounded-2xl px-4 py-2.5 shadow-sm bg-brand-600 text-white rounded-br-md</t>
+        </is>
+      </c>
+      <c r="F24" s="41" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G24" s="41" t="inlineStr">
+        <is>
+          <t>bubble ฝั่งขวา — พื้นหลังสีน้ำเงิน (brand-600)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="41" t="inlineStr">
+        <is>
+          <t>Message Area</t>
+        </is>
+      </c>
+      <c r="B25" s="41" t="inlineStr">
+        <is>
+          <t>Outbound container (flex-end wrapper)</t>
+        </is>
+      </c>
+      <c r="C25" s="41" t="inlineStr">
+        <is>
+          <t>div[class*='justify-end']</t>
+        </is>
+      </c>
+      <c r="D25" s="41" t="inlineStr">
+        <is>
+          <t>div</t>
+        </is>
+      </c>
+      <c r="E25" s="41" t="inlineStr">
+        <is>
+          <t>flex justify-end</t>
+        </is>
+      </c>
+      <c r="F25" s="41" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G25" s="41" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="41" t="inlineStr">
+        <is>
+          <t>Message Area</t>
+        </is>
+      </c>
+      <c r="B26" s="41" t="inlineStr">
+        <is>
+          <t>Message text content</t>
+        </is>
+      </c>
+      <c r="C26" s="41" t="inlineStr">
+        <is>
+          <t>div[class*='whitespace-pre-wrap']</t>
+        </is>
+      </c>
+      <c r="D26" s="41" t="inlineStr">
+        <is>
+          <t>div</t>
+        </is>
+      </c>
+      <c r="E26" s="41" t="inlineStr">
+        <is>
+          <t>whitespace-pre-wrap text-sm leading-relaxed</t>
+        </is>
+      </c>
+      <c r="F26" s="41" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G26" s="41" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="41" t="inlineStr">
+        <is>
+          <t>Message Area</t>
+        </is>
+      </c>
+      <c r="B27" s="41" t="inlineStr">
+        <is>
+          <t>Message timestamp (11:35 น.)</t>
+        </is>
+      </c>
+      <c r="C27" s="41" t="inlineStr">
+        <is>
+          <t>div[class*='text-[11px]'][class*='text-slate-400']</t>
+        </is>
+      </c>
+      <c r="D27" s="41" t="inlineStr">
+        <is>
+          <t>div</t>
+        </is>
+      </c>
+      <c r="E27" s="41" t="inlineStr">
+        <is>
+          <t>mt-1 px-1 text-[11px] text-slate-400 text-right</t>
+        </is>
+      </c>
+      <c r="F27" s="41" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G27" s="41" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="42" t="inlineStr">
+        <is>
+          <t>Message Area</t>
+        </is>
+      </c>
+      <c r="B28" s="42" t="inlineStr">
+        <is>
+          <t>Inbound bubble (patient)</t>
+        </is>
+      </c>
+      <c r="C28" s="42" t="inlineStr">
+        <is>
+          <t>div[class*='justify-start'] div[class*='rounded-2xl']</t>
+        </is>
+      </c>
+      <c r="D28" s="42" t="inlineStr">
+        <is>
+          <t>div</t>
+        </is>
+      </c>
+      <c r="E28" s="42" t="inlineStr">
+        <is>
+          <t>(opposite of outbound — justify-start)</t>
+        </is>
+      </c>
+      <c r="F28" s="42" t="inlineStr">
+        <is>
+          <t>⚠️ อนุมาน</t>
+        </is>
+      </c>
+      <c r="G28" s="42" t="inlineStr">
+        <is>
+          <t>ยังไม่มี inbound message ในขณะ test — ต้องส่งจาก LIFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ZONE 2 — INPUT AREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="43" t="inlineStr">
+        <is>
+          <t>Input Area</t>
+        </is>
+      </c>
+      <c r="B30" s="43" t="inlineStr">
+        <is>
+          <t>Chat message input</t>
+        </is>
+      </c>
+      <c r="C30" s="43" t="inlineStr">
+        <is>
+          <t>input[placeholder*='พิมพ์ข้อความ']</t>
+        </is>
+      </c>
+      <c r="D30" s="43" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="E30" s="43" t="inlineStr">
+        <is>
+          <t>h-10 flex-1 rounded-lg border border-slate-200 bg-slate-50 px-3.5 text-sm</t>
+        </is>
+      </c>
+      <c r="F30" s="43" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G30" s="43" t="inlineStr">
+        <is>
+          <t>⚠️ เป็น input[type=text] ไม่ใช่ textarea!</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="43" t="inlineStr">
+        <is>
+          <t>Input Area</t>
+        </is>
+      </c>
+      <c r="B31" s="43" t="inlineStr">
+        <is>
+          <t>Send button (icon, square)</t>
+        </is>
+      </c>
+      <c r="C31" s="43" t="inlineStr">
+        <is>
+          <t>button[class*='bg-brand-600'][class*='h-10'][class*='w-10']</t>
+        </is>
+      </c>
+      <c r="D31" s="43" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="E31" s="43" t="inlineStr">
+        <is>
+          <t>flex h-10 w-10 shrink-0 items-center justify-center rounded-lg bg-brand-600 … disabled:opacity-40</t>
+        </is>
+      </c>
+      <c r="F31" s="43" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G31" s="43" t="inlineStr">
+        <is>
+          <t>disabled=true เมื่อ input ว่าง | enabled เมื่อมีข้อความ</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="43" t="inlineStr">
+        <is>
+          <t>Input Area</t>
+        </is>
+      </c>
+      <c r="B32" s="43" t="inlineStr">
+        <is>
+          <t>Attach file (label, not button!)</t>
+        </is>
+      </c>
+      <c r="C32" s="43" t="inlineStr">
+        <is>
+          <t>label[class*='shrink-0'][class*='cursor-pointer']</t>
+        </is>
+      </c>
+      <c r="D32" s="43" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="E32" s="43" t="inlineStr">
+        <is>
+          <t>shrink-0 cursor-pointer</t>
+        </is>
+      </c>
+      <c r="F32" s="43" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G32" s="43" t="inlineStr">
+        <is>
+          <t>⚠️ เป็น &lt;label&gt; ไม่ใช่ &lt;button&gt;! — triggers file input</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="43" t="inlineStr">
+        <is>
+          <t>Input Area</t>
+        </is>
+      </c>
+      <c r="B33" s="43" t="inlineStr">
+        <is>
+          <t>File input (hidden)</t>
+        </is>
+      </c>
+      <c r="C33" s="43" t="inlineStr">
+        <is>
+          <t>input[type='file']</t>
+        </is>
+      </c>
+      <c r="D33" s="43" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="E33" s="43" t="inlineStr">
+        <is>
+          <t>hidden</t>
+        </is>
+      </c>
+      <c r="F33" s="43" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G33" s="43" t="inlineStr">
+        <is>
+          <t>display:none — trigger ผ่าน label</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="44" t="inlineStr">
+        <is>
+          <t>Input Area</t>
+        </is>
+      </c>
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>Mic button</t>
+        </is>
+      </c>
+      <c r="C34" s="44" t="inlineStr">
+        <is>
+          <t>(ไม่มีใน UI ปัจจุบัน)</t>
+        </is>
+      </c>
+      <c r="D34" s="44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E34" s="44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F34" s="44" t="inlineStr">
+        <is>
+          <t>❌ ไม่มี</t>
+        </is>
+      </c>
+      <c r="G34" s="44" t="inlineStr">
+        <is>
+          <t>ไม่พบ mic button ใน DOM — send disabled/enabled แทน</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CONFIRM DIALOG (Close Encounter)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="46" t="inlineStr">
+        <is>
+          <t>Dialog</t>
+        </is>
+      </c>
+      <c r="B36" s="46" t="inlineStr">
+        <is>
+          <t>Dialog container</t>
+        </is>
+      </c>
+      <c r="C36" s="46" t="inlineStr">
+        <is>
+          <t>[role='dialog']</t>
+        </is>
+      </c>
+      <c r="D36" s="46" t="inlineStr">
+        <is>
+          <t>div</t>
+        </is>
+      </c>
+      <c r="E36" s="46" t="inlineStr">
+        <is>
+          <t>relative flex max-h-[90vh] w-full flex-col rounded-2xl bg-white shadow-2xl ring-1 … animate-fade-in max-w-md</t>
+        </is>
+      </c>
+      <c r="F36" s="46" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G36" s="46" t="inlineStr">
+        <is>
+          <t>role='dialog' aria-modal='true'</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="46" t="inlineStr">
+        <is>
+          <t>Dialog</t>
+        </is>
+      </c>
+      <c r="B37" s="46" t="inlineStr">
+        <is>
+          <t>Dialog title</t>
+        </is>
+      </c>
+      <c r="C37" s="46" t="inlineStr">
+        <is>
+          <t>[role='dialog'] h3</t>
+        </is>
+      </c>
+      <c r="D37" s="46" t="inlineStr">
+        <is>
+          <t>h3</t>
+        </is>
+      </c>
+      <c r="E37" s="46" t="inlineStr">
+        <is>
+          <t>text-lg font-bold tracking-tight text-slate-900</t>
+        </is>
+      </c>
+      <c r="F37" s="46" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G37" s="46" t="inlineStr">
+        <is>
+          <t>ข้อความ: 'ยืนยันการจบ Session'</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="46" t="inlineStr">
+        <is>
+          <t>Dialog</t>
+        </is>
+      </c>
+      <c r="B38" s="46" t="inlineStr">
+        <is>
+          <t>Cancel button</t>
+        </is>
+      </c>
+      <c r="C38" s="46" t="inlineStr">
+        <is>
+          <t>[role='dialog'] button:has-text('ยกเลิก')</t>
+        </is>
+      </c>
+      <c r="D38" s="46" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="E38" s="46" t="inlineStr">
+        <is>
+          <t>… bg-white hover:bg-slate-50 … text-slate-700 border-slate-200 … h-9 px-4 text-sm …</t>
+        </is>
+      </c>
+      <c r="F38" s="46" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G38" s="46" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="46" t="inlineStr">
+        <is>
+          <t>Dialog</t>
+        </is>
+      </c>
+      <c r="B39" s="46" t="inlineStr">
+        <is>
+          <t>Confirm button (ยืนยันจบ Session)</t>
+        </is>
+      </c>
+      <c r="C39" s="46" t="inlineStr">
+        <is>
+          <t>[role='dialog'] button:has-text('ยืนยันจบ Session')</t>
+        </is>
+      </c>
+      <c r="D39" s="46" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="E39" s="46" t="inlineStr">
+        <is>
+          <t>… bg-danger-600 hover:bg-danger-500 … text-white … h-9 px-4 text-sm …</t>
+        </is>
+      </c>
+      <c r="F39" s="46" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G39" s="46" t="inlineStr">
+        <is>
+          <t>สีแดง bg-danger-600</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AFTER CLOSE ENCOUNTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="47" t="inlineStr">
+        <is>
+          <t>Post-Close</t>
+        </is>
+      </c>
+      <c r="B41" s="47" t="inlineStr">
+        <is>
+          <t>Queue card CLOSED badge</t>
+        </is>
+      </c>
+      <c r="C41" s="47" t="inlineStr">
+        <is>
+          <t>span:has-text('CLOSED')</t>
+        </is>
+      </c>
+      <c r="D41" s="47" t="inlineStr">
+        <is>
+          <t>span</t>
+        </is>
+      </c>
+      <c r="E41" s="47" t="inlineStr">
+        <is>
+          <t>(status badge in Zone 1)</t>
+        </is>
+      </c>
+      <c r="F41" s="47" t="inlineStr">
+        <is>
+          <t>✅ ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G41" s="47" t="inlineStr">
+        <is>
+          <t>ปรากฏใน Zone 1 หลังปิด encounter</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="42" t="inlineStr">
+        <is>
+          <t>Post-Close</t>
+        </is>
+      </c>
+      <c r="B42" s="42" t="inlineStr">
+        <is>
+          <t>Chat input blocked</t>
+        </is>
+      </c>
+      <c r="C42" s="42" t="inlineStr">
+        <is>
+          <t>input[placeholder*='พิมพ์ข้อความ'][disabled]</t>
+        </is>
+      </c>
+      <c r="D42" s="42" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="E42" s="42" t="inlineStr">
+        <is>
+          <t>(disabled attribute)</t>
+        </is>
+      </c>
+      <c r="F42" s="42" t="inlineStr">
+        <is>
+          <t>⚠️ ตรวจเพิ่ม</t>
+        </is>
+      </c>
+      <c r="G42" s="42" t="inlineStr">
+        <is>
+          <t>อาจ disabled หรือ hidden ขึ้นกับ implementation</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A35:G35"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A29:G29"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>